<commit_message>
feat: sync updated user data and final model reports
</commit_message>
<xml_diff>
--- a/ml/data/raw_transactions_user1.xlsx
+++ b/ml/data/raw_transactions_user1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\朱冠勳\Desktop\專題相關\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\朱冠勳\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F5C0C86-6312-4A12-938B-CC91B972FBA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D51FF09E-FF28-4440-BC80-8AD1C6CFDFF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{AD095DF6-AEFA-42CA-AFFD-E1E5631CA533}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="6">
   <si>
     <t>time_stamp</t>
   </si>
@@ -51,6 +51,10 @@
   </si>
   <si>
     <t>Expense</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Income</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -438,7 +442,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DF334D9-454E-4A17-AF44-7CD391DE71B0}">
-  <dimension ref="A1:D281"/>
+  <dimension ref="A1:D286"/>
   <sheetFormatPr defaultRowHeight="16.149999999999999" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
@@ -644,17 +648,17 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A14" s="1">
-        <v>45291</v>
+        <v>45292</v>
       </c>
       <c r="B14" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C14">
-        <v>659</v>
+        <v>10000</v>
       </c>
       <c r="D14">
         <f t="shared" si="0"/>
-        <v>-2069</v>
+        <v>8590</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.45">
@@ -665,11 +669,11 @@
         <v>4</v>
       </c>
       <c r="C15">
-        <v>100</v>
+        <v>659</v>
       </c>
       <c r="D15">
         <f t="shared" si="0"/>
-        <v>-2169</v>
+        <v>7931</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.45">
@@ -680,26 +684,26 @@
         <v>4</v>
       </c>
       <c r="C16">
-        <v>250</v>
+        <v>100</v>
       </c>
       <c r="D16">
         <f t="shared" si="0"/>
-        <v>-2419</v>
+        <v>7831</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A17" s="1">
-        <v>45289</v>
+        <v>45291</v>
       </c>
       <c r="B17" t="s">
         <v>4</v>
       </c>
       <c r="C17">
-        <v>47</v>
+        <v>250</v>
       </c>
       <c r="D17">
         <f t="shared" si="0"/>
-        <v>-2466</v>
+        <v>7581</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.45">
@@ -710,26 +714,26 @@
         <v>4</v>
       </c>
       <c r="C18">
-        <v>118</v>
+        <v>47</v>
       </c>
       <c r="D18">
         <f t="shared" si="0"/>
-        <v>-2584</v>
+        <v>7534</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A19" s="1">
-        <v>45288</v>
+        <v>45289</v>
       </c>
       <c r="B19" t="s">
         <v>4</v>
       </c>
       <c r="C19">
-        <v>153</v>
+        <v>118</v>
       </c>
       <c r="D19">
         <f t="shared" si="0"/>
-        <v>-2737</v>
+        <v>7416</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.45">
@@ -740,26 +744,26 @@
         <v>4</v>
       </c>
       <c r="C20">
-        <v>108</v>
+        <v>153</v>
       </c>
       <c r="D20">
         <f t="shared" si="0"/>
-        <v>-2845</v>
+        <v>7263</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A21" s="1">
-        <v>45287</v>
+        <v>45288</v>
       </c>
       <c r="B21" t="s">
         <v>4</v>
       </c>
       <c r="C21">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="D21">
         <f t="shared" si="0"/>
-        <v>-2945</v>
+        <v>7155</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.45">
@@ -770,26 +774,26 @@
         <v>4</v>
       </c>
       <c r="C22">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="D22">
         <f t="shared" si="0"/>
-        <v>-3008</v>
+        <v>7055</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A23" s="1">
-        <v>45286</v>
+        <v>45287</v>
       </c>
       <c r="B23" t="s">
         <v>4</v>
       </c>
       <c r="C23">
-        <v>30</v>
+        <v>63</v>
       </c>
       <c r="D23">
         <f t="shared" si="0"/>
-        <v>-3038</v>
+        <v>6992</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.45">
@@ -800,41 +804,41 @@
         <v>4</v>
       </c>
       <c r="C24">
-        <v>110</v>
+        <v>30</v>
       </c>
       <c r="D24">
         <f t="shared" si="0"/>
-        <v>-3148</v>
+        <v>6962</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A25" s="1">
-        <v>45285</v>
+        <v>45286</v>
       </c>
       <c r="B25" t="s">
         <v>4</v>
       </c>
       <c r="C25">
-        <v>85</v>
+        <v>110</v>
       </c>
       <c r="D25">
         <f t="shared" si="0"/>
-        <v>-3233</v>
+        <v>6852</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A26" s="1">
-        <v>45284</v>
+        <v>45285</v>
       </c>
       <c r="B26" t="s">
         <v>4</v>
       </c>
       <c r="C26">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="D26">
         <f t="shared" si="0"/>
-        <v>-3333</v>
+        <v>6767</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.45">
@@ -845,41 +849,41 @@
         <v>4</v>
       </c>
       <c r="C27">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D27">
         <f t="shared" si="0"/>
-        <v>-3434</v>
+        <v>6667</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A28" s="1">
-        <v>45283</v>
+        <v>45284</v>
       </c>
       <c r="B28" t="s">
         <v>4</v>
       </c>
       <c r="C28">
-        <v>588</v>
+        <v>101</v>
       </c>
       <c r="D28">
         <f t="shared" si="0"/>
-        <v>-4022</v>
+        <v>6566</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A29" s="1">
-        <v>45282</v>
+        <v>45283</v>
       </c>
       <c r="B29" t="s">
         <v>4</v>
       </c>
       <c r="C29">
-        <v>100</v>
+        <v>588</v>
       </c>
       <c r="D29">
         <f t="shared" si="0"/>
-        <v>-4122</v>
+        <v>5978</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.45">
@@ -890,11 +894,11 @@
         <v>4</v>
       </c>
       <c r="C30">
-        <v>380</v>
+        <v>100</v>
       </c>
       <c r="D30">
         <f t="shared" si="0"/>
-        <v>-4502</v>
+        <v>5878</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.45">
@@ -905,11 +909,11 @@
         <v>4</v>
       </c>
       <c r="C31">
-        <v>50</v>
+        <v>380</v>
       </c>
       <c r="D31">
         <f t="shared" si="0"/>
-        <v>-4552</v>
+        <v>5498</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.45">
@@ -920,26 +924,26 @@
         <v>4</v>
       </c>
       <c r="C32">
-        <v>130</v>
+        <v>50</v>
       </c>
       <c r="D32">
         <f t="shared" si="0"/>
-        <v>-4682</v>
+        <v>5448</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A33" s="1">
-        <v>45281</v>
+        <v>45282</v>
       </c>
       <c r="B33" t="s">
         <v>4</v>
       </c>
       <c r="C33">
-        <v>461</v>
+        <v>130</v>
       </c>
       <c r="D33">
         <f t="shared" si="0"/>
-        <v>-5143</v>
+        <v>5318</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.45">
@@ -950,26 +954,26 @@
         <v>4</v>
       </c>
       <c r="C34">
-        <v>155</v>
+        <v>461</v>
       </c>
       <c r="D34">
         <f t="shared" si="0"/>
-        <v>-5298</v>
+        <v>4857</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A35" s="1">
-        <v>45280</v>
+        <v>45281</v>
       </c>
       <c r="B35" t="s">
         <v>4</v>
       </c>
       <c r="C35">
-        <v>100</v>
+        <v>155</v>
       </c>
       <c r="D35">
         <f t="shared" si="0"/>
-        <v>-5398</v>
+        <v>4702</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.45">
@@ -980,26 +984,26 @@
         <v>4</v>
       </c>
       <c r="C36">
-        <v>260</v>
+        <v>100</v>
       </c>
       <c r="D36">
         <f t="shared" si="0"/>
-        <v>-5658</v>
+        <v>4602</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A37" s="1">
-        <v>45279</v>
+        <v>45280</v>
       </c>
       <c r="B37" t="s">
         <v>4</v>
       </c>
       <c r="C37">
-        <v>99</v>
+        <v>260</v>
       </c>
       <c r="D37">
         <f t="shared" si="0"/>
-        <v>-5757</v>
+        <v>4342</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.45">
@@ -1010,11 +1014,11 @@
         <v>4</v>
       </c>
       <c r="C38">
-        <v>52</v>
+        <v>99</v>
       </c>
       <c r="D38">
         <f t="shared" si="0"/>
-        <v>-5809</v>
+        <v>4243</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.45">
@@ -1025,26 +1029,26 @@
         <v>4</v>
       </c>
       <c r="C39">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="D39">
         <f t="shared" si="0"/>
-        <v>-5854</v>
+        <v>4191</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A40" s="1">
-        <v>45278</v>
+        <v>45279</v>
       </c>
       <c r="B40" t="s">
         <v>4</v>
       </c>
       <c r="C40">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="D40">
         <f t="shared" si="0"/>
-        <v>-5879</v>
+        <v>4146</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.45">
@@ -1055,11 +1059,11 @@
         <v>4</v>
       </c>
       <c r="C41">
-        <v>115</v>
+        <v>25</v>
       </c>
       <c r="D41">
         <f t="shared" si="0"/>
-        <v>-5994</v>
+        <v>4121</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.45">
@@ -1070,11 +1074,11 @@
         <v>4</v>
       </c>
       <c r="C42">
-        <v>90</v>
+        <v>115</v>
       </c>
       <c r="D42">
         <f t="shared" si="0"/>
-        <v>-6084</v>
+        <v>4006</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.45">
@@ -1085,26 +1089,26 @@
         <v>4</v>
       </c>
       <c r="C43">
-        <v>74</v>
+        <v>90</v>
       </c>
       <c r="D43">
         <f t="shared" si="0"/>
-        <v>-6158</v>
+        <v>3916</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A44" s="1">
-        <v>45277</v>
+        <v>45278</v>
       </c>
       <c r="B44" t="s">
         <v>4</v>
       </c>
       <c r="C44">
-        <v>25</v>
+        <v>74</v>
       </c>
       <c r="D44">
         <f t="shared" si="0"/>
-        <v>-6183</v>
+        <v>3842</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.45">
@@ -1115,11 +1119,11 @@
         <v>4</v>
       </c>
       <c r="C45">
-        <v>510</v>
+        <v>25</v>
       </c>
       <c r="D45">
         <f t="shared" si="0"/>
-        <v>-6693</v>
+        <v>3817</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.45">
@@ -1130,11 +1134,11 @@
         <v>4</v>
       </c>
       <c r="C46">
-        <v>200</v>
+        <v>510</v>
       </c>
       <c r="D46">
         <f t="shared" si="0"/>
-        <v>-6893</v>
+        <v>3307</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.45">
@@ -1145,26 +1149,26 @@
         <v>4</v>
       </c>
       <c r="C47">
-        <v>130</v>
+        <v>200</v>
       </c>
       <c r="D47">
         <f t="shared" si="0"/>
-        <v>-7023</v>
+        <v>3107</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A48" s="1">
-        <v>45276</v>
+        <v>45277</v>
       </c>
       <c r="B48" t="s">
         <v>4</v>
       </c>
       <c r="C48">
-        <v>890</v>
+        <v>130</v>
       </c>
       <c r="D48">
         <f t="shared" si="0"/>
-        <v>-7913</v>
+        <v>2977</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.45">
@@ -1175,11 +1179,11 @@
         <v>4</v>
       </c>
       <c r="C49">
-        <v>90</v>
+        <v>890</v>
       </c>
       <c r="D49">
         <f t="shared" si="0"/>
-        <v>-8003</v>
+        <v>2087</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.45">
@@ -1190,41 +1194,41 @@
         <v>4</v>
       </c>
       <c r="C50">
-        <v>335</v>
+        <v>90</v>
       </c>
       <c r="D50">
         <f t="shared" si="0"/>
-        <v>-8338</v>
+        <v>1997</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A51" s="1">
-        <v>45275</v>
+        <v>45276</v>
       </c>
       <c r="B51" t="s">
         <v>4</v>
       </c>
       <c r="C51">
-        <v>104</v>
+        <v>335</v>
       </c>
       <c r="D51">
         <f t="shared" si="0"/>
-        <v>-8442</v>
+        <v>1662</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A52" s="1">
-        <v>45274</v>
+        <v>45275</v>
       </c>
       <c r="B52" t="s">
         <v>4</v>
       </c>
       <c r="C52">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D52">
         <f t="shared" si="0"/>
-        <v>-8542</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.45">
@@ -1235,26 +1239,26 @@
         <v>4</v>
       </c>
       <c r="C53">
-        <v>155</v>
+        <v>100</v>
       </c>
       <c r="D53">
         <f t="shared" si="0"/>
-        <v>-8697</v>
+        <v>1458</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A54" s="1">
-        <v>45273</v>
+        <v>45274</v>
       </c>
       <c r="B54" t="s">
         <v>4</v>
       </c>
       <c r="C54">
-        <v>90</v>
+        <v>155</v>
       </c>
       <c r="D54">
         <f t="shared" si="0"/>
-        <v>-8787</v>
+        <v>1303</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.45">
@@ -1265,26 +1269,26 @@
         <v>4</v>
       </c>
       <c r="C55">
-        <v>280</v>
+        <v>90</v>
       </c>
       <c r="D55">
         <f t="shared" si="0"/>
-        <v>-9067</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A56" s="1">
-        <v>45272</v>
+        <v>45273</v>
       </c>
       <c r="B56" t="s">
         <v>4</v>
       </c>
       <c r="C56">
-        <v>75</v>
+        <v>280</v>
       </c>
       <c r="D56">
         <f t="shared" si="0"/>
-        <v>-9142</v>
+        <v>933</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.45">
@@ -1295,11 +1299,11 @@
         <v>4</v>
       </c>
       <c r="C57">
-        <v>160</v>
+        <v>75</v>
       </c>
       <c r="D57">
         <f t="shared" si="0"/>
-        <v>-9302</v>
+        <v>858</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.45">
@@ -1310,11 +1314,11 @@
         <v>4</v>
       </c>
       <c r="C58">
-        <v>68</v>
+        <v>160</v>
       </c>
       <c r="D58">
         <f t="shared" si="0"/>
-        <v>-9370</v>
+        <v>698</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.45">
@@ -1325,26 +1329,26 @@
         <v>4</v>
       </c>
       <c r="C59">
-        <v>130</v>
+        <v>68</v>
       </c>
       <c r="D59">
         <f t="shared" si="0"/>
-        <v>-9500</v>
+        <v>630</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A60" s="1">
-        <v>45271</v>
+        <v>45272</v>
       </c>
       <c r="B60" t="s">
         <v>4</v>
       </c>
       <c r="C60">
-        <v>80</v>
+        <v>130</v>
       </c>
       <c r="D60">
         <f t="shared" si="0"/>
-        <v>-9580</v>
+        <v>500</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.45">
@@ -1355,11 +1359,11 @@
         <v>4</v>
       </c>
       <c r="C61">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="D61">
         <f t="shared" si="0"/>
-        <v>-9680</v>
+        <v>420</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.45">
@@ -1370,11 +1374,11 @@
         <v>4</v>
       </c>
       <c r="C62">
-        <v>45</v>
+        <v>100</v>
       </c>
       <c r="D62">
         <f t="shared" si="0"/>
-        <v>-9725</v>
+        <v>320</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.45">
@@ -1385,26 +1389,26 @@
         <v>4</v>
       </c>
       <c r="C63">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="D63">
         <f t="shared" si="0"/>
-        <v>-9755</v>
+        <v>275</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A64" s="1">
-        <v>45270</v>
+        <v>45271</v>
       </c>
       <c r="B64" t="s">
         <v>4</v>
       </c>
       <c r="C64">
-        <v>69</v>
+        <v>30</v>
       </c>
       <c r="D64">
         <f t="shared" si="0"/>
-        <v>-9824</v>
+        <v>245</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.45">
@@ -1415,26 +1419,26 @@
         <v>4</v>
       </c>
       <c r="C65">
-        <v>23</v>
+        <v>69</v>
       </c>
       <c r="D65">
         <f t="shared" si="0"/>
-        <v>-9847</v>
+        <v>176</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A66" s="1">
-        <v>45269</v>
+        <v>45270</v>
       </c>
       <c r="B66" t="s">
         <v>4</v>
       </c>
       <c r="C66">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="D66">
         <f t="shared" si="0"/>
-        <v>-9892</v>
+        <v>153</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.45">
@@ -1445,11 +1449,11 @@
         <v>4</v>
       </c>
       <c r="C67">
-        <v>100</v>
+        <v>45</v>
       </c>
       <c r="D67">
         <f t="shared" si="0"/>
-        <v>-9992</v>
+        <v>108</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.45">
@@ -1460,11 +1464,11 @@
         <v>4</v>
       </c>
       <c r="C68">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="D68">
         <f t="shared" ref="D68:D131" si="1">IF(B68="Income",D67+C68,D67-C68)</f>
-        <v>-10007</v>
+        <v>8</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.45">
@@ -1475,26 +1479,26 @@
         <v>4</v>
       </c>
       <c r="C69">
-        <v>190</v>
+        <v>15</v>
       </c>
       <c r="D69">
         <f t="shared" si="1"/>
-        <v>-10197</v>
+        <v>-7</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A70" s="1">
-        <v>45268</v>
+        <v>45269</v>
       </c>
       <c r="B70" t="s">
         <v>4</v>
       </c>
       <c r="C70">
-        <v>49</v>
+        <v>190</v>
       </c>
       <c r="D70">
         <f t="shared" si="1"/>
-        <v>-10246</v>
+        <v>-197</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.45">
@@ -1505,11 +1509,11 @@
         <v>4</v>
       </c>
       <c r="C71">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="D71">
         <f t="shared" si="1"/>
-        <v>-10306</v>
+        <v>-246</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.45">
@@ -1520,26 +1524,26 @@
         <v>4</v>
       </c>
       <c r="C72">
-        <v>95</v>
+        <v>60</v>
       </c>
       <c r="D72">
         <f t="shared" si="1"/>
-        <v>-10401</v>
+        <v>-306</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A73" s="1">
-        <v>45267</v>
+        <v>45268</v>
       </c>
       <c r="B73" t="s">
         <v>4</v>
       </c>
       <c r="C73">
-        <v>68</v>
+        <v>95</v>
       </c>
       <c r="D73">
         <f t="shared" si="1"/>
-        <v>-10469</v>
+        <v>-401</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.45">
@@ -1550,11 +1554,11 @@
         <v>4</v>
       </c>
       <c r="C74">
-        <v>45</v>
+        <v>68</v>
       </c>
       <c r="D74">
         <f t="shared" si="1"/>
-        <v>-10514</v>
+        <v>-469</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.45">
@@ -1565,26 +1569,26 @@
         <v>4</v>
       </c>
       <c r="C75">
-        <v>178</v>
+        <v>45</v>
       </c>
       <c r="D75">
         <f t="shared" si="1"/>
-        <v>-10692</v>
+        <v>-514</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A76" s="1">
-        <v>45266</v>
+        <v>45267</v>
       </c>
       <c r="B76" t="s">
         <v>4</v>
       </c>
       <c r="C76">
-        <v>45</v>
+        <v>178</v>
       </c>
       <c r="D76">
         <f t="shared" si="1"/>
-        <v>-10737</v>
+        <v>-692</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.45">
@@ -1595,11 +1599,11 @@
         <v>4</v>
       </c>
       <c r="C77">
-        <v>100</v>
+        <v>45</v>
       </c>
       <c r="D77">
         <f t="shared" si="1"/>
-        <v>-10837</v>
+        <v>-737</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.45">
@@ -1614,22 +1618,22 @@
       </c>
       <c r="D78">
         <f t="shared" si="1"/>
-        <v>-10937</v>
+        <v>-837</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A79" s="1">
-        <v>45265</v>
+        <v>45266</v>
       </c>
       <c r="B79" t="s">
         <v>4</v>
       </c>
       <c r="C79">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="D79">
         <f t="shared" si="1"/>
-        <v>-11027</v>
+        <v>-937</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.45">
@@ -1640,11 +1644,11 @@
         <v>4</v>
       </c>
       <c r="C80">
-        <v>110</v>
+        <v>90</v>
       </c>
       <c r="D80">
         <f t="shared" si="1"/>
-        <v>-11137</v>
+        <v>-1027</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.45">
@@ -1655,11 +1659,11 @@
         <v>4</v>
       </c>
       <c r="C81">
-        <v>25</v>
+        <v>110</v>
       </c>
       <c r="D81">
         <f t="shared" si="1"/>
-        <v>-11162</v>
+        <v>-1137</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.45">
@@ -1670,26 +1674,26 @@
         <v>4</v>
       </c>
       <c r="C82">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D82">
         <f t="shared" si="1"/>
-        <v>-11182</v>
+        <v>-1162</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A83" s="1">
-        <v>45264</v>
+        <v>45265</v>
       </c>
       <c r="B83" t="s">
         <v>4</v>
       </c>
       <c r="C83">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="D83">
         <f t="shared" si="1"/>
-        <v>-11242</v>
+        <v>-1182</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.45">
@@ -1700,41 +1704,41 @@
         <v>4</v>
       </c>
       <c r="C84">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="D84">
         <f t="shared" si="1"/>
-        <v>-11267</v>
+        <v>-1242</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A85" s="1">
-        <v>45263</v>
+        <v>45264</v>
       </c>
       <c r="B85" t="s">
         <v>4</v>
       </c>
       <c r="C85">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="D85">
         <f t="shared" si="1"/>
-        <v>-11367</v>
+        <v>-1267</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A86" s="1">
-        <v>45261</v>
+        <v>45263</v>
       </c>
       <c r="B86" t="s">
         <v>4</v>
       </c>
       <c r="C86">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="D86">
         <f t="shared" si="1"/>
-        <v>-11397</v>
+        <v>-1367</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.45">
@@ -1745,11 +1749,11 @@
         <v>4</v>
       </c>
       <c r="C87">
-        <v>110</v>
+        <v>30</v>
       </c>
       <c r="D87">
         <f t="shared" si="1"/>
-        <v>-11507</v>
+        <v>-1397</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.45">
@@ -1760,56 +1764,56 @@
         <v>4</v>
       </c>
       <c r="C88">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="D88">
         <f t="shared" si="1"/>
-        <v>-11607</v>
+        <v>-1507</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A89" s="1">
-        <v>45260</v>
+        <v>45261</v>
       </c>
       <c r="B89" t="s">
         <v>4</v>
       </c>
       <c r="C89">
-        <v>163</v>
+        <v>100</v>
       </c>
       <c r="D89">
         <f t="shared" si="1"/>
-        <v>-11770</v>
+        <v>-1607</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A90" s="1">
-        <v>45259</v>
+        <v>45261</v>
       </c>
       <c r="B90" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C90">
-        <v>235</v>
+        <v>10000</v>
       </c>
       <c r="D90">
         <f t="shared" si="1"/>
-        <v>-12005</v>
+        <v>8393</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A91" s="1">
-        <v>45259</v>
+        <v>45260</v>
       </c>
       <c r="B91" t="s">
         <v>4</v>
       </c>
       <c r="C91">
-        <v>65</v>
+        <v>163</v>
       </c>
       <c r="D91">
         <f t="shared" si="1"/>
-        <v>-12070</v>
+        <v>8230</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.45">
@@ -1820,41 +1824,41 @@
         <v>4</v>
       </c>
       <c r="C92">
-        <v>99</v>
+        <v>235</v>
       </c>
       <c r="D92">
         <f t="shared" si="1"/>
-        <v>-12169</v>
+        <v>7995</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A93" s="1">
-        <v>45258</v>
+        <v>45259</v>
       </c>
       <c r="B93" t="s">
         <v>4</v>
       </c>
       <c r="C93">
-        <v>150</v>
+        <v>65</v>
       </c>
       <c r="D93">
         <f t="shared" si="1"/>
-        <v>-12319</v>
+        <v>7930</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A94" s="1">
-        <v>45258</v>
+        <v>45259</v>
       </c>
       <c r="B94" t="s">
         <v>4</v>
       </c>
       <c r="C94">
-        <v>180</v>
+        <v>99</v>
       </c>
       <c r="D94">
         <f t="shared" si="1"/>
-        <v>-12499</v>
+        <v>7831</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.45">
@@ -1865,11 +1869,11 @@
         <v>4</v>
       </c>
       <c r="C95">
-        <v>110</v>
+        <v>150</v>
       </c>
       <c r="D95">
         <f t="shared" si="1"/>
-        <v>-12609</v>
+        <v>7681</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.45">
@@ -1880,41 +1884,41 @@
         <v>4</v>
       </c>
       <c r="C96">
-        <v>36</v>
+        <v>180</v>
       </c>
       <c r="D96">
         <f t="shared" si="1"/>
-        <v>-12645</v>
+        <v>7501</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A97" s="1">
-        <v>45257</v>
+        <v>45258</v>
       </c>
       <c r="B97" t="s">
         <v>4</v>
       </c>
       <c r="C97">
-        <v>268</v>
+        <v>110</v>
       </c>
       <c r="D97">
         <f t="shared" si="1"/>
-        <v>-12913</v>
+        <v>7391</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A98" s="1">
-        <v>45257</v>
+        <v>45258</v>
       </c>
       <c r="B98" t="s">
         <v>4</v>
       </c>
       <c r="C98">
-        <v>588</v>
+        <v>36</v>
       </c>
       <c r="D98">
         <f t="shared" si="1"/>
-        <v>-13501</v>
+        <v>7355</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.45">
@@ -1925,11 +1929,11 @@
         <v>4</v>
       </c>
       <c r="C99">
-        <v>25</v>
+        <v>268</v>
       </c>
       <c r="D99">
         <f t="shared" si="1"/>
-        <v>-13526</v>
+        <v>7087</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.45">
@@ -1940,86 +1944,86 @@
         <v>4</v>
       </c>
       <c r="C100">
-        <v>69</v>
+        <v>588</v>
       </c>
       <c r="D100">
         <f t="shared" si="1"/>
-        <v>-13595</v>
+        <v>6499</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A101" s="1">
-        <v>45256</v>
+        <v>45257</v>
       </c>
       <c r="B101" t="s">
         <v>4</v>
       </c>
       <c r="C101">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="D101">
         <f t="shared" si="1"/>
-        <v>-13695</v>
+        <v>6474</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A102" s="1">
-        <v>45256</v>
+        <v>45257</v>
       </c>
       <c r="B102" t="s">
         <v>4</v>
       </c>
       <c r="C102">
-        <v>260</v>
+        <v>69</v>
       </c>
       <c r="D102">
         <f t="shared" si="1"/>
-        <v>-13955</v>
+        <v>6405</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A103" s="1">
-        <v>45254</v>
+        <v>45256</v>
       </c>
       <c r="B103" t="s">
         <v>4</v>
       </c>
       <c r="C103">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="D103">
         <f t="shared" si="1"/>
-        <v>-14020</v>
+        <v>6305</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A104" s="1">
-        <v>45253</v>
+        <v>45256</v>
       </c>
       <c r="B104" t="s">
         <v>4</v>
       </c>
       <c r="C104">
-        <v>471</v>
+        <v>260</v>
       </c>
       <c r="D104">
         <f t="shared" si="1"/>
-        <v>-14491</v>
+        <v>6045</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A105" s="1">
-        <v>45253</v>
+        <v>45254</v>
       </c>
       <c r="B105" t="s">
         <v>4</v>
       </c>
       <c r="C105">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="D105">
         <f t="shared" si="1"/>
-        <v>-14536</v>
+        <v>5980</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.45">
@@ -2030,16 +2034,16 @@
         <v>4</v>
       </c>
       <c r="C106">
-        <v>130</v>
+        <v>471</v>
       </c>
       <c r="D106">
         <f t="shared" si="1"/>
-        <v>-14666</v>
+        <v>5509</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A107" s="1">
-        <v>45252</v>
+        <v>45253</v>
       </c>
       <c r="B107" t="s">
         <v>4</v>
@@ -2049,22 +2053,22 @@
       </c>
       <c r="D107">
         <f t="shared" si="1"/>
-        <v>-14711</v>
+        <v>5464</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A108" s="1">
-        <v>45252</v>
+        <v>45253</v>
       </c>
       <c r="B108" t="s">
         <v>4</v>
       </c>
       <c r="C108">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="D108">
         <f t="shared" si="1"/>
-        <v>-14811</v>
+        <v>5334</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.45">
@@ -2075,11 +2079,11 @@
         <v>4</v>
       </c>
       <c r="C109">
-        <v>95</v>
+        <v>45</v>
       </c>
       <c r="D109">
         <f t="shared" si="1"/>
-        <v>-14906</v>
+        <v>5289</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.45">
@@ -2090,11 +2094,11 @@
         <v>4</v>
       </c>
       <c r="C110">
-        <v>190</v>
+        <v>100</v>
       </c>
       <c r="D110">
         <f t="shared" si="1"/>
-        <v>-15096</v>
+        <v>5189</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.45">
@@ -2105,41 +2109,41 @@
         <v>4</v>
       </c>
       <c r="C111">
-        <v>20</v>
+        <v>95</v>
       </c>
       <c r="D111">
         <f t="shared" si="1"/>
-        <v>-15116</v>
+        <v>5094</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A112" s="1">
-        <v>45251</v>
+        <v>45252</v>
       </c>
       <c r="B112" t="s">
         <v>4</v>
       </c>
       <c r="C112">
-        <v>1600</v>
+        <v>190</v>
       </c>
       <c r="D112">
         <f t="shared" si="1"/>
-        <v>-16716</v>
+        <v>4904</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A113" s="1">
-        <v>45251</v>
+        <v>45252</v>
       </c>
       <c r="B113" t="s">
         <v>4</v>
       </c>
       <c r="C113">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="D113">
         <f t="shared" si="1"/>
-        <v>-16786</v>
+        <v>4884</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.45">
@@ -2150,11 +2154,11 @@
         <v>4</v>
       </c>
       <c r="C114">
-        <v>47</v>
+        <v>1600</v>
       </c>
       <c r="D114">
         <f t="shared" si="1"/>
-        <v>-16833</v>
+        <v>3284</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.45">
@@ -2165,101 +2169,101 @@
         <v>4</v>
       </c>
       <c r="C115">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="D115">
         <f t="shared" si="1"/>
-        <v>-16878</v>
+        <v>3214</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A116" s="1">
-        <v>45249</v>
+        <v>45251</v>
       </c>
       <c r="B116" t="s">
         <v>4</v>
       </c>
       <c r="C116">
-        <v>139</v>
+        <v>47</v>
       </c>
       <c r="D116">
         <f t="shared" si="1"/>
-        <v>-17017</v>
+        <v>3167</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A117" s="1">
-        <v>45249</v>
+        <v>45251</v>
       </c>
       <c r="B117" t="s">
         <v>4</v>
       </c>
       <c r="C117">
-        <v>100</v>
+        <v>45</v>
       </c>
       <c r="D117">
         <f t="shared" si="1"/>
-        <v>-17117</v>
+        <v>3122</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A118" s="1">
-        <v>45247</v>
+        <v>45249</v>
       </c>
       <c r="B118" t="s">
         <v>4</v>
       </c>
       <c r="C118">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="D118">
         <f t="shared" si="1"/>
-        <v>-17217</v>
+        <v>2983</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A119" s="1">
-        <v>45247</v>
+        <v>45249</v>
       </c>
       <c r="B119" t="s">
         <v>4</v>
       </c>
       <c r="C119">
-        <v>47</v>
+        <v>100</v>
       </c>
       <c r="D119">
         <f t="shared" si="1"/>
-        <v>-17264</v>
+        <v>2883</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A120" s="1">
-        <v>45246</v>
+        <v>45247</v>
       </c>
       <c r="B120" t="s">
         <v>4</v>
       </c>
       <c r="C120">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="D120">
         <f t="shared" si="1"/>
-        <v>-17314</v>
+        <v>2783</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A121" s="1">
-        <v>45246</v>
+        <v>45247</v>
       </c>
       <c r="B121" t="s">
         <v>4</v>
       </c>
       <c r="C121">
-        <v>200</v>
+        <v>47</v>
       </c>
       <c r="D121">
         <f t="shared" si="1"/>
-        <v>-17514</v>
+        <v>2736</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.45">
@@ -2270,41 +2274,41 @@
         <v>4</v>
       </c>
       <c r="C122">
-        <v>110</v>
+        <v>50</v>
       </c>
       <c r="D122">
         <f t="shared" si="1"/>
-        <v>-17624</v>
+        <v>2686</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A123" s="1">
-        <v>45245</v>
+        <v>45246</v>
       </c>
       <c r="B123" t="s">
         <v>4</v>
       </c>
       <c r="C123">
-        <v>680</v>
+        <v>200</v>
       </c>
       <c r="D123">
         <f t="shared" si="1"/>
-        <v>-18304</v>
+        <v>2486</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A124" s="1">
-        <v>45245</v>
+        <v>45246</v>
       </c>
       <c r="B124" t="s">
         <v>4</v>
       </c>
       <c r="C124">
-        <v>55</v>
+        <v>110</v>
       </c>
       <c r="D124">
         <f t="shared" si="1"/>
-        <v>-18359</v>
+        <v>2376</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.45">
@@ -2315,11 +2319,11 @@
         <v>4</v>
       </c>
       <c r="C125">
-        <v>55</v>
+        <v>680</v>
       </c>
       <c r="D125">
         <f t="shared" si="1"/>
-        <v>-18414</v>
+        <v>1696</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.45">
@@ -2330,11 +2334,11 @@
         <v>4</v>
       </c>
       <c r="C126">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="D126">
         <f t="shared" si="1"/>
-        <v>-18494</v>
+        <v>1641</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.45">
@@ -2345,41 +2349,41 @@
         <v>4</v>
       </c>
       <c r="C127">
-        <v>130</v>
+        <v>55</v>
       </c>
       <c r="D127">
         <f t="shared" si="1"/>
-        <v>-18624</v>
+        <v>1586</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A128" s="1">
-        <v>45244</v>
+        <v>45245</v>
       </c>
       <c r="B128" t="s">
         <v>4</v>
       </c>
       <c r="C128">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="D128">
         <f t="shared" si="1"/>
-        <v>-18681</v>
+        <v>1506</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A129" s="1">
-        <v>45244</v>
+        <v>45245</v>
       </c>
       <c r="B129" t="s">
         <v>4</v>
       </c>
       <c r="C129">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="D129">
         <f t="shared" si="1"/>
-        <v>-18781</v>
+        <v>1376</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.45">
@@ -2390,61 +2394,61 @@
         <v>4</v>
       </c>
       <c r="C130">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="D130">
         <f t="shared" si="1"/>
-        <v>-18826</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A131" s="1">
-        <v>45243</v>
+        <v>45244</v>
       </c>
       <c r="B131" t="s">
         <v>4</v>
       </c>
       <c r="C131">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="D131">
         <f t="shared" si="1"/>
-        <v>-18906</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A132" s="1">
-        <v>45243</v>
+        <v>45244</v>
       </c>
       <c r="B132" t="s">
         <v>4</v>
       </c>
       <c r="C132">
-        <v>100</v>
+        <v>45</v>
       </c>
       <c r="D132">
         <f t="shared" ref="D132:D195" si="2">IF(B132="Income",D131+C132,D131-C132)</f>
-        <v>-19006</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A133" s="1">
-        <v>45241</v>
+        <v>45243</v>
       </c>
       <c r="B133" t="s">
         <v>4</v>
       </c>
       <c r="C133">
-        <v>164</v>
+        <v>80</v>
       </c>
       <c r="D133">
         <f t="shared" si="2"/>
-        <v>-19170</v>
+        <v>1094</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A134" s="1">
-        <v>45241</v>
+        <v>45243</v>
       </c>
       <c r="B134" t="s">
         <v>4</v>
@@ -2454,7 +2458,7 @@
       </c>
       <c r="D134">
         <f t="shared" si="2"/>
-        <v>-19270</v>
+        <v>994</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.45">
@@ -2465,11 +2469,11 @@
         <v>4</v>
       </c>
       <c r="C135">
-        <v>25</v>
+        <v>164</v>
       </c>
       <c r="D135">
         <f t="shared" si="2"/>
-        <v>-19295</v>
+        <v>830</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.45">
@@ -2484,7 +2488,7 @@
       </c>
       <c r="D136">
         <f t="shared" si="2"/>
-        <v>-19395</v>
+        <v>730</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.45">
@@ -2495,56 +2499,56 @@
         <v>4</v>
       </c>
       <c r="C137">
-        <v>600</v>
+        <v>25</v>
       </c>
       <c r="D137">
         <f t="shared" si="2"/>
-        <v>-19995</v>
+        <v>705</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A138" s="1">
-        <v>45240</v>
+        <v>45241</v>
       </c>
       <c r="B138" t="s">
         <v>4</v>
       </c>
       <c r="C138">
-        <v>236</v>
+        <v>100</v>
       </c>
       <c r="D138">
         <f t="shared" si="2"/>
-        <v>-20231</v>
+        <v>605</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A139" s="1">
-        <v>45239</v>
+        <v>45241</v>
       </c>
       <c r="B139" t="s">
         <v>4</v>
       </c>
       <c r="C139">
-        <v>55</v>
+        <v>600</v>
       </c>
       <c r="D139">
         <f t="shared" si="2"/>
-        <v>-20286</v>
+        <v>5</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A140" s="1">
-        <v>45239</v>
+        <v>45240</v>
       </c>
       <c r="B140" t="s">
         <v>4</v>
       </c>
       <c r="C140">
-        <v>138</v>
+        <v>236</v>
       </c>
       <c r="D140">
         <f t="shared" si="2"/>
-        <v>-20424</v>
+        <v>-231</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.45">
@@ -2555,11 +2559,11 @@
         <v>4</v>
       </c>
       <c r="C141">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="D141">
         <f t="shared" si="2"/>
-        <v>-20457</v>
+        <v>-286</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.45">
@@ -2570,71 +2574,71 @@
         <v>4</v>
       </c>
       <c r="C142">
-        <v>16</v>
+        <v>138</v>
       </c>
       <c r="D142">
         <f t="shared" si="2"/>
-        <v>-20473</v>
+        <v>-424</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A143" s="1">
-        <v>45238</v>
+        <v>45239</v>
       </c>
       <c r="B143" t="s">
         <v>4</v>
       </c>
       <c r="C143">
-        <v>110</v>
+        <v>33</v>
       </c>
       <c r="D143">
         <f t="shared" si="2"/>
-        <v>-20583</v>
+        <v>-457</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A144" s="1">
-        <v>45238</v>
+        <v>45239</v>
       </c>
       <c r="B144" t="s">
         <v>4</v>
       </c>
       <c r="C144">
-        <v>60</v>
+        <v>16</v>
       </c>
       <c r="D144">
         <f t="shared" si="2"/>
-        <v>-20643</v>
+        <v>-473</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A145" s="1">
-        <v>45237</v>
+        <v>45238</v>
       </c>
       <c r="B145" t="s">
         <v>4</v>
       </c>
       <c r="C145">
-        <v>20</v>
+        <v>110</v>
       </c>
       <c r="D145">
         <f t="shared" si="2"/>
-        <v>-20663</v>
+        <v>-583</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A146" s="1">
-        <v>45237</v>
+        <v>45238</v>
       </c>
       <c r="B146" t="s">
         <v>4</v>
       </c>
       <c r="C146">
-        <v>99</v>
+        <v>60</v>
       </c>
       <c r="D146">
         <f t="shared" si="2"/>
-        <v>-20762</v>
+        <v>-643</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.45">
@@ -2645,11 +2649,11 @@
         <v>4</v>
       </c>
       <c r="C147">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D147">
         <f t="shared" si="2"/>
-        <v>-20787</v>
+        <v>-663</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.45">
@@ -2660,41 +2664,41 @@
         <v>4</v>
       </c>
       <c r="C148">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D148">
         <f t="shared" si="2"/>
-        <v>-20887</v>
+        <v>-762</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A149" s="1">
-        <v>45236</v>
+        <v>45237</v>
       </c>
       <c r="B149" t="s">
         <v>4</v>
       </c>
       <c r="C149">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="D149">
         <f t="shared" si="2"/>
-        <v>-20942</v>
+        <v>-787</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A150" s="1">
-        <v>45236</v>
+        <v>45237</v>
       </c>
       <c r="B150" t="s">
         <v>4</v>
       </c>
       <c r="C150">
-        <v>55</v>
+        <v>100</v>
       </c>
       <c r="D150">
         <f t="shared" si="2"/>
-        <v>-20997</v>
+        <v>-887</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.45">
@@ -2705,11 +2709,11 @@
         <v>4</v>
       </c>
       <c r="C151">
-        <v>100</v>
+        <v>55</v>
       </c>
       <c r="D151">
         <f t="shared" si="2"/>
-        <v>-21097</v>
+        <v>-942</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.45">
@@ -2720,56 +2724,56 @@
         <v>4</v>
       </c>
       <c r="C152">
-        <v>190</v>
+        <v>55</v>
       </c>
       <c r="D152">
         <f t="shared" si="2"/>
-        <v>-21287</v>
+        <v>-997</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A153" s="1">
-        <v>45234</v>
+        <v>45236</v>
       </c>
       <c r="B153" t="s">
         <v>4</v>
       </c>
       <c r="C153">
-        <v>79</v>
+        <v>100</v>
       </c>
       <c r="D153">
         <f t="shared" si="2"/>
-        <v>-21366</v>
+        <v>-1097</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A154" s="1">
-        <v>45233</v>
+        <v>45236</v>
       </c>
       <c r="B154" t="s">
         <v>4</v>
       </c>
       <c r="C154">
-        <v>27</v>
+        <v>190</v>
       </c>
       <c r="D154">
         <f t="shared" si="2"/>
-        <v>-21393</v>
+        <v>-1287</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A155" s="1">
-        <v>45233</v>
+        <v>45234</v>
       </c>
       <c r="B155" t="s">
         <v>4</v>
       </c>
       <c r="C155">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="D155">
         <f t="shared" si="2"/>
-        <v>-21503</v>
+        <v>-1366</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.45">
@@ -2780,41 +2784,41 @@
         <v>4</v>
       </c>
       <c r="C156">
-        <v>100</v>
+        <v>27</v>
       </c>
       <c r="D156">
         <f t="shared" si="2"/>
-        <v>-21603</v>
+        <v>-1393</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A157" s="1">
-        <v>45232</v>
+        <v>45233</v>
       </c>
       <c r="B157" t="s">
         <v>4</v>
       </c>
       <c r="C157">
-        <v>35</v>
+        <v>110</v>
       </c>
       <c r="D157">
         <f t="shared" si="2"/>
-        <v>-21638</v>
+        <v>-1503</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A158" s="1">
-        <v>45232</v>
+        <v>45233</v>
       </c>
       <c r="B158" t="s">
         <v>4</v>
       </c>
       <c r="C158">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="D158">
         <f t="shared" si="2"/>
-        <v>-21658</v>
+        <v>-1603</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.45">
@@ -2825,11 +2829,11 @@
         <v>4</v>
       </c>
       <c r="C159">
-        <v>110</v>
+        <v>35</v>
       </c>
       <c r="D159">
         <f t="shared" si="2"/>
-        <v>-21768</v>
+        <v>-1638</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.45">
@@ -2840,41 +2844,41 @@
         <v>4</v>
       </c>
       <c r="C160">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="D160">
         <f t="shared" si="2"/>
-        <v>-21848</v>
+        <v>-1658</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A161" s="1">
-        <v>45231</v>
+        <v>45232</v>
       </c>
       <c r="B161" t="s">
         <v>4</v>
       </c>
       <c r="C161">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="D161">
         <f t="shared" si="2"/>
-        <v>-21938</v>
+        <v>-1768</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A162" s="1">
-        <v>45231</v>
+        <v>45232</v>
       </c>
       <c r="B162" t="s">
         <v>4</v>
       </c>
       <c r="C162">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="D162">
         <f t="shared" si="2"/>
-        <v>-22012</v>
+        <v>-1848</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.45">
@@ -2885,56 +2889,56 @@
         <v>4</v>
       </c>
       <c r="C163">
-        <v>164</v>
+        <v>90</v>
       </c>
       <c r="D163">
         <f t="shared" si="2"/>
-        <v>-22176</v>
+        <v>-1938</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A164" s="1">
-        <v>45230</v>
+        <v>45231</v>
       </c>
       <c r="B164" t="s">
         <v>4</v>
       </c>
       <c r="C164">
-        <v>267</v>
+        <v>74</v>
       </c>
       <c r="D164">
         <f t="shared" si="2"/>
-        <v>-22443</v>
+        <v>-2012</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A165" s="1">
-        <v>45230</v>
+        <v>45231</v>
       </c>
       <c r="B165" t="s">
         <v>4</v>
       </c>
       <c r="C165">
-        <v>124</v>
+        <v>164</v>
       </c>
       <c r="D165">
         <f t="shared" si="2"/>
-        <v>-22567</v>
+        <v>-2176</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A166" s="1">
-        <v>45230</v>
+        <v>45231</v>
       </c>
       <c r="B166" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C166">
-        <v>162</v>
+        <v>10000</v>
       </c>
       <c r="D166">
         <f t="shared" si="2"/>
-        <v>-22729</v>
+        <v>7824</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.45">
@@ -2945,11 +2949,11 @@
         <v>4</v>
       </c>
       <c r="C167">
-        <v>85</v>
+        <v>267</v>
       </c>
       <c r="D167">
         <f t="shared" si="2"/>
-        <v>-22814</v>
+        <v>7557</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.45">
@@ -2960,11 +2964,11 @@
         <v>4</v>
       </c>
       <c r="C168">
-        <v>50</v>
+        <v>124</v>
       </c>
       <c r="D168">
         <f t="shared" si="2"/>
-        <v>-22864</v>
+        <v>7433</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.45">
@@ -2975,11 +2979,11 @@
         <v>4</v>
       </c>
       <c r="C169">
-        <v>500</v>
+        <v>162</v>
       </c>
       <c r="D169">
         <f t="shared" si="2"/>
-        <v>-23364</v>
+        <v>7271</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.45">
@@ -2990,11 +2994,11 @@
         <v>4</v>
       </c>
       <c r="C170">
-        <v>55</v>
+        <v>85</v>
       </c>
       <c r="D170">
         <f t="shared" si="2"/>
-        <v>-23419</v>
+        <v>7186</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.45">
@@ -3005,11 +3009,11 @@
         <v>4</v>
       </c>
       <c r="C171">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="D171">
         <f t="shared" si="2"/>
-        <v>-23489</v>
+        <v>7136</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.45">
@@ -3020,11 +3024,11 @@
         <v>4</v>
       </c>
       <c r="C172">
-        <v>385</v>
+        <v>500</v>
       </c>
       <c r="D172">
         <f t="shared" si="2"/>
-        <v>-23874</v>
+        <v>6636</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.45">
@@ -3035,101 +3039,101 @@
         <v>4</v>
       </c>
       <c r="C173">
-        <v>100</v>
+        <v>55</v>
       </c>
       <c r="D173">
         <f t="shared" si="2"/>
-        <v>-23974</v>
+        <v>6581</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A174" s="1">
-        <v>45227</v>
+        <v>45230</v>
       </c>
       <c r="B174" t="s">
         <v>4</v>
       </c>
       <c r="C174">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="D174">
         <f t="shared" si="2"/>
-        <v>-24074</v>
+        <v>6511</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A175" s="1">
-        <v>45227</v>
+        <v>45230</v>
       </c>
       <c r="B175" t="s">
         <v>4</v>
       </c>
       <c r="C175">
-        <v>590</v>
+        <v>385</v>
       </c>
       <c r="D175">
         <f t="shared" si="2"/>
-        <v>-24664</v>
+        <v>6126</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A176" s="1">
-        <v>45227</v>
+        <v>45230</v>
       </c>
       <c r="B176" t="s">
         <v>4</v>
       </c>
       <c r="C176">
-        <v>208</v>
+        <v>100</v>
       </c>
       <c r="D176">
         <f t="shared" si="2"/>
-        <v>-24872</v>
+        <v>6026</v>
       </c>
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A177" s="1">
-        <v>45226</v>
+        <v>45227</v>
       </c>
       <c r="B177" t="s">
         <v>4</v>
       </c>
       <c r="C177">
-        <v>17</v>
+        <v>100</v>
       </c>
       <c r="D177">
         <f t="shared" si="2"/>
-        <v>-24889</v>
+        <v>5926</v>
       </c>
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A178" s="1">
-        <v>45226</v>
+        <v>45227</v>
       </c>
       <c r="B178" t="s">
         <v>4</v>
       </c>
       <c r="C178">
-        <v>160</v>
+        <v>590</v>
       </c>
       <c r="D178">
         <f t="shared" si="2"/>
-        <v>-25049</v>
+        <v>5336</v>
       </c>
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A179" s="1">
-        <v>45226</v>
+        <v>45227</v>
       </c>
       <c r="B179" t="s">
         <v>4</v>
       </c>
       <c r="C179">
-        <v>80</v>
+        <v>208</v>
       </c>
       <c r="D179">
         <f t="shared" si="2"/>
-        <v>-25129</v>
+        <v>5128</v>
       </c>
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.45">
@@ -3140,11 +3144,11 @@
         <v>4</v>
       </c>
       <c r="C180">
-        <v>100</v>
+        <v>17</v>
       </c>
       <c r="D180">
         <f t="shared" si="2"/>
-        <v>-25229</v>
+        <v>5111</v>
       </c>
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.45">
@@ -3155,16 +3159,16 @@
         <v>4</v>
       </c>
       <c r="C181">
-        <v>27</v>
+        <v>160</v>
       </c>
       <c r="D181">
         <f t="shared" si="2"/>
-        <v>-25256</v>
+        <v>4951</v>
       </c>
     </row>
     <row r="182" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A182" s="1">
-        <v>45225</v>
+        <v>45226</v>
       </c>
       <c r="B182" t="s">
         <v>4</v>
@@ -3174,37 +3178,37 @@
       </c>
       <c r="D182">
         <f t="shared" si="2"/>
-        <v>-25336</v>
+        <v>4871</v>
       </c>
     </row>
     <row r="183" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A183" s="1">
-        <v>45225</v>
+        <v>45226</v>
       </c>
       <c r="B183" t="s">
         <v>4</v>
       </c>
       <c r="C183">
-        <v>45</v>
+        <v>100</v>
       </c>
       <c r="D183">
         <f t="shared" si="2"/>
-        <v>-25381</v>
+        <v>4771</v>
       </c>
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A184" s="1">
-        <v>45225</v>
+        <v>45226</v>
       </c>
       <c r="B184" t="s">
         <v>4</v>
       </c>
       <c r="C184">
-        <v>150</v>
+        <v>27</v>
       </c>
       <c r="D184">
         <f t="shared" si="2"/>
-        <v>-25531</v>
+        <v>4744</v>
       </c>
     </row>
     <row r="185" spans="1:4" x14ac:dyDescent="0.45">
@@ -3215,56 +3219,56 @@
         <v>4</v>
       </c>
       <c r="C185">
-        <v>16</v>
+        <v>80</v>
       </c>
       <c r="D185">
         <f t="shared" si="2"/>
-        <v>-25547</v>
+        <v>4664</v>
       </c>
     </row>
     <row r="186" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A186" s="1">
-        <v>45224</v>
+        <v>45225</v>
       </c>
       <c r="B186" t="s">
         <v>4</v>
       </c>
       <c r="C186">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="D186">
         <f t="shared" si="2"/>
-        <v>-25602</v>
+        <v>4619</v>
       </c>
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A187" s="1">
-        <v>45224</v>
+        <v>45225</v>
       </c>
       <c r="B187" t="s">
         <v>4</v>
       </c>
       <c r="C187">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="D187">
         <f t="shared" si="2"/>
-        <v>-25652</v>
+        <v>4469</v>
       </c>
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A188" s="1">
-        <v>45224</v>
+        <v>45225</v>
       </c>
       <c r="B188" t="s">
         <v>4</v>
       </c>
       <c r="C188">
-        <v>90</v>
+        <v>16</v>
       </c>
       <c r="D188">
         <f t="shared" si="2"/>
-        <v>-25742</v>
+        <v>4453</v>
       </c>
     </row>
     <row r="189" spans="1:4" x14ac:dyDescent="0.45">
@@ -3275,206 +3279,206 @@
         <v>4</v>
       </c>
       <c r="C189">
-        <v>95</v>
+        <v>55</v>
       </c>
       <c r="D189">
         <f t="shared" si="2"/>
-        <v>-25837</v>
+        <v>4398</v>
       </c>
     </row>
     <row r="190" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A190" s="1">
-        <v>45223</v>
+        <v>45224</v>
       </c>
       <c r="B190" t="s">
         <v>4</v>
       </c>
       <c r="C190">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="D190">
         <f t="shared" si="2"/>
-        <v>-25867</v>
+        <v>4348</v>
       </c>
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A191" s="1">
-        <v>45223</v>
+        <v>45224</v>
       </c>
       <c r="B191" t="s">
         <v>4</v>
       </c>
       <c r="C191">
-        <v>25</v>
+        <v>90</v>
       </c>
       <c r="D191">
         <f t="shared" si="2"/>
-        <v>-25892</v>
+        <v>4258</v>
       </c>
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A192" s="1">
-        <v>45223</v>
+        <v>45224</v>
       </c>
       <c r="B192" t="s">
         <v>4</v>
       </c>
       <c r="C192">
-        <v>140</v>
+        <v>95</v>
       </c>
       <c r="D192">
         <f t="shared" si="2"/>
-        <v>-26032</v>
+        <v>4163</v>
       </c>
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A193" s="1">
-        <v>45222</v>
+        <v>45223</v>
       </c>
       <c r="B193" t="s">
         <v>4</v>
       </c>
       <c r="C193">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="D193">
         <f t="shared" si="2"/>
-        <v>-26112</v>
+        <v>4133</v>
       </c>
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A194" s="1">
-        <v>45222</v>
+        <v>45223</v>
       </c>
       <c r="B194" t="s">
         <v>4</v>
       </c>
       <c r="C194">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="D194">
         <f t="shared" si="2"/>
-        <v>-26212</v>
+        <v>4108</v>
       </c>
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A195" s="1">
-        <v>45222</v>
+        <v>45223</v>
       </c>
       <c r="B195" t="s">
         <v>4</v>
       </c>
       <c r="C195">
-        <v>50</v>
+        <v>140</v>
       </c>
       <c r="D195">
         <f t="shared" si="2"/>
-        <v>-26262</v>
+        <v>3968</v>
       </c>
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A196" s="1">
-        <v>45221</v>
+        <v>45222</v>
       </c>
       <c r="B196" t="s">
         <v>4</v>
       </c>
       <c r="C196">
-        <v>450</v>
+        <v>80</v>
       </c>
       <c r="D196">
         <f t="shared" ref="D196:D259" si="3">IF(B196="Income",D195+C196,D195-C196)</f>
-        <v>-26712</v>
+        <v>3888</v>
       </c>
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A197" s="1">
-        <v>45220</v>
+        <v>45222</v>
       </c>
       <c r="B197" t="s">
         <v>4</v>
       </c>
       <c r="C197">
-        <v>600</v>
+        <v>100</v>
       </c>
       <c r="D197">
         <f t="shared" si="3"/>
-        <v>-27312</v>
+        <v>3788</v>
       </c>
     </row>
     <row r="198" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A198" s="1">
-        <v>45220</v>
+        <v>45222</v>
       </c>
       <c r="B198" t="s">
         <v>4</v>
       </c>
       <c r="C198">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D198">
         <f t="shared" si="3"/>
-        <v>-27512</v>
+        <v>3738</v>
       </c>
     </row>
     <row r="199" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A199" s="1">
-        <v>45220</v>
+        <v>45221</v>
       </c>
       <c r="B199" t="s">
         <v>4</v>
       </c>
       <c r="C199">
-        <v>100</v>
+        <v>450</v>
       </c>
       <c r="D199">
         <f t="shared" si="3"/>
-        <v>-27612</v>
+        <v>3288</v>
       </c>
     </row>
     <row r="200" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A200" s="1">
-        <v>45219</v>
+        <v>45220</v>
       </c>
       <c r="B200" t="s">
         <v>4</v>
       </c>
       <c r="C200">
-        <v>36</v>
+        <v>600</v>
       </c>
       <c r="D200">
         <f t="shared" si="3"/>
-        <v>-27648</v>
+        <v>2688</v>
       </c>
     </row>
     <row r="201" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A201" s="1">
-        <v>45219</v>
+        <v>45220</v>
       </c>
       <c r="B201" t="s">
         <v>4</v>
       </c>
       <c r="C201">
-        <v>85</v>
+        <v>200</v>
       </c>
       <c r="D201">
         <f t="shared" si="3"/>
-        <v>-27733</v>
+        <v>2488</v>
       </c>
     </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A202" s="1">
-        <v>45219</v>
+        <v>45220</v>
       </c>
       <c r="B202" t="s">
         <v>4</v>
       </c>
       <c r="C202">
-        <v>45</v>
+        <v>100</v>
       </c>
       <c r="D202">
         <f t="shared" si="3"/>
-        <v>-27778</v>
+        <v>2388</v>
       </c>
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.45">
@@ -3485,311 +3489,311 @@
         <v>4</v>
       </c>
       <c r="C203">
-        <v>97</v>
+        <v>36</v>
       </c>
       <c r="D203">
         <f t="shared" si="3"/>
-        <v>-27875</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A204" s="1">
-        <v>45218</v>
+        <v>45219</v>
       </c>
       <c r="B204" t="s">
         <v>4</v>
       </c>
       <c r="C204">
-        <v>38</v>
+        <v>85</v>
       </c>
       <c r="D204">
         <f t="shared" si="3"/>
-        <v>-27913</v>
+        <v>2267</v>
       </c>
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A205" s="1">
-        <v>45218</v>
+        <v>45219</v>
       </c>
       <c r="B205" t="s">
         <v>4</v>
       </c>
       <c r="C205">
-        <v>200</v>
+        <v>45</v>
       </c>
       <c r="D205">
         <f t="shared" si="3"/>
-        <v>-28113</v>
+        <v>2222</v>
       </c>
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A206" s="1">
-        <v>45217</v>
+        <v>45219</v>
       </c>
       <c r="B206" t="s">
         <v>4</v>
       </c>
       <c r="C206">
-        <v>55</v>
+        <v>97</v>
       </c>
       <c r="D206">
         <f t="shared" si="3"/>
-        <v>-28168</v>
+        <v>2125</v>
       </c>
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A207" s="1">
-        <v>45217</v>
+        <v>45218</v>
       </c>
       <c r="B207" t="s">
         <v>4</v>
       </c>
       <c r="C207">
-        <v>110</v>
+        <v>38</v>
       </c>
       <c r="D207">
         <f t="shared" si="3"/>
-        <v>-28278</v>
+        <v>2087</v>
       </c>
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A208" s="1">
-        <v>45216</v>
+        <v>45218</v>
       </c>
       <c r="B208" t="s">
         <v>4</v>
       </c>
       <c r="C208">
-        <v>77</v>
+        <v>200</v>
       </c>
       <c r="D208">
         <f t="shared" si="3"/>
-        <v>-28355</v>
+        <v>1887</v>
       </c>
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A209" s="1">
-        <v>45216</v>
+        <v>45217</v>
       </c>
       <c r="B209" t="s">
         <v>4</v>
       </c>
       <c r="C209">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="D209">
         <f t="shared" si="3"/>
-        <v>-28425</v>
+        <v>1832</v>
       </c>
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A210" s="1">
-        <v>45215</v>
+        <v>45217</v>
       </c>
       <c r="B210" t="s">
         <v>4</v>
       </c>
       <c r="C210">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="D210">
         <f t="shared" si="3"/>
-        <v>-28525</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A211" s="1">
-        <v>45215</v>
+        <v>45216</v>
       </c>
       <c r="B211" t="s">
         <v>4</v>
       </c>
       <c r="C211">
-        <v>120</v>
+        <v>77</v>
       </c>
       <c r="D211">
         <f t="shared" si="3"/>
-        <v>-28645</v>
+        <v>1645</v>
       </c>
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A212" s="1">
-        <v>45214</v>
+        <v>45216</v>
       </c>
       <c r="B212" t="s">
         <v>4</v>
       </c>
       <c r="C212">
-        <v>150</v>
+        <v>70</v>
       </c>
       <c r="D212">
         <f t="shared" si="3"/>
-        <v>-28795</v>
+        <v>1575</v>
       </c>
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A213" s="1">
-        <v>45213</v>
+        <v>45215</v>
       </c>
       <c r="B213" t="s">
         <v>4</v>
       </c>
       <c r="C213">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="D213">
         <f t="shared" si="3"/>
-        <v>-28820</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A214" s="1">
-        <v>45212</v>
+        <v>45215</v>
       </c>
       <c r="B214" t="s">
         <v>4</v>
       </c>
       <c r="C214">
-        <v>65</v>
+        <v>120</v>
       </c>
       <c r="D214">
         <f t="shared" si="3"/>
-        <v>-28885</v>
+        <v>1355</v>
       </c>
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A215" s="1">
-        <v>45212</v>
+        <v>45214</v>
       </c>
       <c r="B215" t="s">
         <v>4</v>
       </c>
       <c r="C215">
-        <v>270</v>
+        <v>150</v>
       </c>
       <c r="D215">
         <f t="shared" si="3"/>
-        <v>-29155</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A216" s="1">
-        <v>45211</v>
+        <v>45213</v>
       </c>
       <c r="B216" t="s">
         <v>4</v>
       </c>
       <c r="C216">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="D216">
         <f t="shared" si="3"/>
-        <v>-29225</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A217" s="1">
-        <v>45211</v>
+        <v>45212</v>
       </c>
       <c r="B217" t="s">
         <v>4</v>
       </c>
       <c r="C217">
-        <v>135</v>
+        <v>65</v>
       </c>
       <c r="D217">
         <f t="shared" si="3"/>
-        <v>-29360</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A218" s="1">
-        <v>45210</v>
+        <v>45212</v>
       </c>
       <c r="B218" t="s">
         <v>4</v>
       </c>
       <c r="C218">
-        <v>55</v>
+        <v>270</v>
       </c>
       <c r="D218">
         <f t="shared" si="3"/>
-        <v>-29415</v>
+        <v>845</v>
       </c>
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A219" s="1">
-        <v>45210</v>
+        <v>45211</v>
       </c>
       <c r="B219" t="s">
         <v>4</v>
       </c>
       <c r="C219">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="D219">
         <f t="shared" si="3"/>
-        <v>-29465</v>
+        <v>775</v>
       </c>
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A220" s="1">
-        <v>45210</v>
+        <v>45211</v>
       </c>
       <c r="B220" t="s">
         <v>4</v>
       </c>
       <c r="C220">
-        <v>30</v>
+        <v>135</v>
       </c>
       <c r="D220">
         <f t="shared" si="3"/>
-        <v>-29495</v>
+        <v>640</v>
       </c>
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A221" s="1">
-        <v>45209</v>
+        <v>45210</v>
       </c>
       <c r="B221" t="s">
         <v>4</v>
       </c>
       <c r="C221">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="D221">
         <f t="shared" si="3"/>
-        <v>-29540</v>
+        <v>585</v>
       </c>
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A222" s="1">
-        <v>45209</v>
+        <v>45210</v>
       </c>
       <c r="B222" t="s">
         <v>4</v>
       </c>
       <c r="C222">
-        <v>145</v>
+        <v>50</v>
       </c>
       <c r="D222">
         <f t="shared" si="3"/>
-        <v>-29685</v>
+        <v>535</v>
       </c>
     </row>
     <row r="223" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A223" s="1">
-        <v>45209</v>
+        <v>45210</v>
       </c>
       <c r="B223" t="s">
         <v>4</v>
       </c>
       <c r="C223">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="D223">
         <f t="shared" si="3"/>
-        <v>-29785</v>
+        <v>505</v>
       </c>
     </row>
     <row r="224" spans="1:4" x14ac:dyDescent="0.45">
@@ -3800,56 +3804,56 @@
         <v>4</v>
       </c>
       <c r="C224">
-        <v>185</v>
+        <v>45</v>
       </c>
       <c r="D224">
         <f t="shared" si="3"/>
-        <v>-29970</v>
+        <v>460</v>
       </c>
     </row>
     <row r="225" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A225" s="1">
-        <v>45208</v>
+        <v>45209</v>
       </c>
       <c r="B225" t="s">
         <v>4</v>
       </c>
       <c r="C225">
-        <v>50</v>
+        <v>145</v>
       </c>
       <c r="D225">
         <f t="shared" si="3"/>
-        <v>-30020</v>
+        <v>315</v>
       </c>
     </row>
     <row r="226" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A226" s="1">
-        <v>45208</v>
+        <v>45209</v>
       </c>
       <c r="B226" t="s">
         <v>4</v>
       </c>
       <c r="C226">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="D226">
         <f t="shared" si="3"/>
-        <v>-30220</v>
+        <v>215</v>
       </c>
     </row>
     <row r="227" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A227" s="1">
-        <v>45208</v>
+        <v>45209</v>
       </c>
       <c r="B227" t="s">
         <v>4</v>
       </c>
       <c r="C227">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="D227">
         <f t="shared" si="3"/>
-        <v>-30409</v>
+        <v>30</v>
       </c>
     </row>
     <row r="228" spans="1:4" x14ac:dyDescent="0.45">
@@ -3860,191 +3864,191 @@
         <v>4</v>
       </c>
       <c r="C228">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="D228">
         <f t="shared" si="3"/>
-        <v>-30509</v>
+        <v>-20</v>
       </c>
     </row>
     <row r="229" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A229" s="1">
-        <v>45205</v>
+        <v>45208</v>
       </c>
       <c r="B229" t="s">
         <v>4</v>
       </c>
       <c r="C229">
-        <v>775</v>
+        <v>200</v>
       </c>
       <c r="D229">
         <f t="shared" si="3"/>
-        <v>-31284</v>
+        <v>-220</v>
       </c>
     </row>
     <row r="230" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A230" s="1">
-        <v>45205</v>
+        <v>45208</v>
       </c>
       <c r="B230" t="s">
         <v>4</v>
       </c>
       <c r="C230">
-        <v>90</v>
+        <v>189</v>
       </c>
       <c r="D230">
         <f t="shared" si="3"/>
-        <v>-31374</v>
+        <v>-409</v>
       </c>
     </row>
     <row r="231" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A231" s="1">
-        <v>45204</v>
+        <v>45208</v>
       </c>
       <c r="B231" t="s">
         <v>4</v>
       </c>
       <c r="C231">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D231">
         <f t="shared" si="3"/>
-        <v>-31494</v>
+        <v>-509</v>
       </c>
     </row>
     <row r="232" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A232" s="1">
-        <v>45204</v>
+        <v>45205</v>
       </c>
       <c r="B232" t="s">
         <v>4</v>
       </c>
       <c r="C232">
-        <v>135</v>
+        <v>775</v>
       </c>
       <c r="D232">
         <f t="shared" si="3"/>
-        <v>-31629</v>
+        <v>-1284</v>
       </c>
     </row>
     <row r="233" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A233" s="1">
-        <v>45203</v>
+        <v>45205</v>
       </c>
       <c r="B233" t="s">
         <v>4</v>
       </c>
       <c r="C233">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="D233">
         <f t="shared" si="3"/>
-        <v>-31659</v>
+        <v>-1374</v>
       </c>
     </row>
     <row r="234" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A234" s="1">
-        <v>45203</v>
+        <v>45204</v>
       </c>
       <c r="B234" t="s">
         <v>4</v>
       </c>
       <c r="C234">
-        <v>250</v>
+        <v>120</v>
       </c>
       <c r="D234">
         <f t="shared" si="3"/>
-        <v>-31909</v>
+        <v>-1494</v>
       </c>
     </row>
     <row r="235" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A235" s="1">
-        <v>45202</v>
+        <v>45204</v>
       </c>
       <c r="B235" t="s">
         <v>4</v>
       </c>
       <c r="C235">
-        <v>518</v>
+        <v>135</v>
       </c>
       <c r="D235">
         <f t="shared" si="3"/>
-        <v>-32427</v>
+        <v>-1629</v>
       </c>
     </row>
     <row r="236" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A236" s="1">
-        <v>45202</v>
+        <v>45203</v>
       </c>
       <c r="B236" t="s">
         <v>4</v>
       </c>
       <c r="C236">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D236">
         <f t="shared" si="3"/>
-        <v>-32459</v>
+        <v>-1659</v>
       </c>
     </row>
     <row r="237" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A237" s="1">
-        <v>45202</v>
+        <v>45203</v>
       </c>
       <c r="B237" t="s">
         <v>4</v>
       </c>
       <c r="C237">
-        <v>145</v>
+        <v>250</v>
       </c>
       <c r="D237">
         <f t="shared" si="3"/>
-        <v>-32604</v>
+        <v>-1909</v>
       </c>
     </row>
     <row r="238" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A238" s="1">
-        <v>45201</v>
+        <v>45202</v>
       </c>
       <c r="B238" t="s">
         <v>4</v>
       </c>
       <c r="C238">
-        <v>100</v>
+        <v>518</v>
       </c>
       <c r="D238">
         <f t="shared" si="3"/>
-        <v>-32704</v>
+        <v>-2427</v>
       </c>
     </row>
     <row r="239" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A239" s="1">
-        <v>45201</v>
+        <v>45202</v>
       </c>
       <c r="B239" t="s">
         <v>4</v>
       </c>
       <c r="C239">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="D239">
         <f t="shared" si="3"/>
-        <v>-32748</v>
+        <v>-2459</v>
       </c>
     </row>
     <row r="240" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A240" s="1">
-        <v>45201</v>
+        <v>45202</v>
       </c>
       <c r="B240" t="s">
         <v>4</v>
       </c>
       <c r="C240">
-        <v>105</v>
+        <v>145</v>
       </c>
       <c r="D240">
         <f t="shared" si="3"/>
-        <v>-32853</v>
+        <v>-2604</v>
       </c>
     </row>
     <row r="241" spans="1:4" x14ac:dyDescent="0.45">
@@ -4055,586 +4059,586 @@
         <v>4</v>
       </c>
       <c r="C241">
-        <v>55</v>
+        <v>100</v>
       </c>
       <c r="D241">
         <f t="shared" si="3"/>
-        <v>-32908</v>
+        <v>-2704</v>
       </c>
     </row>
     <row r="242" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A242" s="1">
-        <v>45197</v>
+        <v>45201</v>
       </c>
       <c r="B242" t="s">
         <v>4</v>
       </c>
       <c r="C242">
-        <v>100</v>
+        <v>44</v>
       </c>
       <c r="D242">
         <f t="shared" si="3"/>
-        <v>-33008</v>
+        <v>-2748</v>
       </c>
     </row>
     <row r="243" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A243" s="1">
-        <v>45197</v>
+        <v>45201</v>
       </c>
       <c r="B243" t="s">
         <v>4</v>
       </c>
       <c r="C243">
-        <v>45</v>
+        <v>105</v>
       </c>
       <c r="D243">
         <f t="shared" si="3"/>
-        <v>-33053</v>
+        <v>-2853</v>
       </c>
     </row>
     <row r="244" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A244" s="1">
-        <v>45197</v>
+        <v>45201</v>
       </c>
       <c r="B244" t="s">
         <v>4</v>
       </c>
       <c r="C244">
-        <v>177</v>
+        <v>55</v>
       </c>
       <c r="D244">
         <f t="shared" si="3"/>
-        <v>-33230</v>
+        <v>-2908</v>
       </c>
     </row>
     <row r="245" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A245" s="1">
-        <v>45197</v>
+        <v>45200</v>
       </c>
       <c r="B245" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C245">
-        <v>126</v>
+        <v>10000</v>
       </c>
       <c r="D245">
         <f t="shared" si="3"/>
-        <v>-33356</v>
+        <v>7092</v>
       </c>
     </row>
     <row r="246" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A246" s="1">
-        <v>45196</v>
+        <v>45197</v>
       </c>
       <c r="B246" t="s">
         <v>4</v>
       </c>
       <c r="C246">
-        <v>55</v>
+        <v>100</v>
       </c>
       <c r="D246">
         <f t="shared" si="3"/>
-        <v>-33411</v>
+        <v>6992</v>
       </c>
     </row>
     <row r="247" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A247" s="1">
-        <v>45196</v>
+        <v>45197</v>
       </c>
       <c r="B247" t="s">
         <v>4</v>
       </c>
       <c r="C247">
-        <v>95</v>
+        <v>45</v>
       </c>
       <c r="D247">
         <f t="shared" si="3"/>
-        <v>-33506</v>
+        <v>6947</v>
       </c>
     </row>
     <row r="248" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A248" s="1">
-        <v>45196</v>
+        <v>45197</v>
       </c>
       <c r="B248" t="s">
         <v>4</v>
       </c>
       <c r="C248">
-        <v>65</v>
+        <v>177</v>
       </c>
       <c r="D248">
         <f t="shared" si="3"/>
-        <v>-33571</v>
+        <v>6770</v>
       </c>
     </row>
     <row r="249" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A249" s="1">
-        <v>45195</v>
+        <v>45197</v>
       </c>
       <c r="B249" t="s">
         <v>4</v>
       </c>
       <c r="C249">
-        <v>50</v>
+        <v>126</v>
       </c>
       <c r="D249">
         <f t="shared" si="3"/>
-        <v>-33621</v>
+        <v>6644</v>
       </c>
     </row>
     <row r="250" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A250" s="1">
-        <v>45194</v>
+        <v>45196</v>
       </c>
       <c r="B250" t="s">
         <v>4</v>
       </c>
       <c r="C250">
-        <v>730</v>
+        <v>55</v>
       </c>
       <c r="D250">
         <f t="shared" si="3"/>
-        <v>-34351</v>
+        <v>6589</v>
       </c>
     </row>
     <row r="251" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A251" s="1">
-        <v>45191</v>
+        <v>45196</v>
       </c>
       <c r="B251" t="s">
         <v>4</v>
       </c>
       <c r="C251">
-        <v>130</v>
+        <v>95</v>
       </c>
       <c r="D251">
         <f t="shared" si="3"/>
-        <v>-34481</v>
+        <v>6494</v>
       </c>
     </row>
     <row r="252" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A252" s="1">
-        <v>45190</v>
+        <v>45196</v>
       </c>
       <c r="B252" t="s">
         <v>4</v>
       </c>
       <c r="C252">
-        <v>300</v>
+        <v>65</v>
       </c>
       <c r="D252">
         <f t="shared" si="3"/>
-        <v>-34781</v>
+        <v>6429</v>
       </c>
     </row>
     <row r="253" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A253" s="1">
-        <v>45190</v>
+        <v>45195</v>
       </c>
       <c r="B253" t="s">
         <v>4</v>
       </c>
       <c r="C253">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="D253">
         <f t="shared" si="3"/>
-        <v>-34808</v>
+        <v>6379</v>
       </c>
     </row>
     <row r="254" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A254" s="1">
-        <v>45189</v>
+        <v>45194</v>
       </c>
       <c r="B254" t="s">
         <v>4</v>
       </c>
       <c r="C254">
-        <v>55</v>
+        <v>730</v>
       </c>
       <c r="D254">
         <f t="shared" si="3"/>
-        <v>-34863</v>
+        <v>5649</v>
       </c>
     </row>
     <row r="255" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A255" s="1">
-        <v>45189</v>
+        <v>45191</v>
       </c>
       <c r="B255" t="s">
         <v>4</v>
       </c>
       <c r="C255">
-        <v>208</v>
+        <v>130</v>
       </c>
       <c r="D255">
         <f t="shared" si="3"/>
-        <v>-35071</v>
+        <v>5519</v>
       </c>
     </row>
     <row r="256" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A256" s="1">
-        <v>45188</v>
+        <v>45190</v>
       </c>
       <c r="B256" t="s">
         <v>4</v>
       </c>
       <c r="C256">
-        <v>22</v>
+        <v>300</v>
       </c>
       <c r="D256">
         <f t="shared" si="3"/>
-        <v>-35093</v>
+        <v>5219</v>
       </c>
     </row>
     <row r="257" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A257" s="1">
-        <v>45187</v>
+        <v>45190</v>
       </c>
       <c r="B257" t="s">
         <v>4</v>
       </c>
       <c r="C257">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="D257">
         <f t="shared" si="3"/>
-        <v>-35143</v>
+        <v>5192</v>
       </c>
     </row>
     <row r="258" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A258" s="1">
-        <v>45187</v>
+        <v>45189</v>
       </c>
       <c r="B258" t="s">
         <v>4</v>
       </c>
       <c r="C258">
-        <v>110</v>
+        <v>55</v>
       </c>
       <c r="D258">
         <f t="shared" si="3"/>
-        <v>-35253</v>
+        <v>5137</v>
       </c>
     </row>
     <row r="259" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A259" s="1">
-        <v>45187</v>
+        <v>45189</v>
       </c>
       <c r="B259" t="s">
         <v>4</v>
       </c>
       <c r="C259">
-        <v>192</v>
+        <v>208</v>
       </c>
       <c r="D259">
         <f t="shared" si="3"/>
-        <v>-35445</v>
+        <v>4929</v>
       </c>
     </row>
     <row r="260" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A260" s="1">
-        <v>45184</v>
+        <v>45188</v>
       </c>
       <c r="B260" t="s">
         <v>4</v>
       </c>
       <c r="C260">
-        <v>155</v>
+        <v>22</v>
       </c>
       <c r="D260">
-        <f t="shared" ref="D260:D281" si="4">IF(B260="Income",D259+C260,D259-C260)</f>
-        <v>-35600</v>
+        <f t="shared" ref="D260:D286" si="4">IF(B260="Income",D259+C260,D259-C260)</f>
+        <v>4907</v>
       </c>
     </row>
     <row r="261" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A261" s="1">
-        <v>45184</v>
+        <v>45187</v>
       </c>
       <c r="B261" t="s">
         <v>4</v>
       </c>
       <c r="C261">
-        <v>800</v>
+        <v>50</v>
       </c>
       <c r="D261">
         <f t="shared" si="4"/>
-        <v>-36400</v>
+        <v>4857</v>
       </c>
     </row>
     <row r="262" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A262" s="1">
-        <v>45183</v>
+        <v>45187</v>
       </c>
       <c r="B262" t="s">
         <v>4</v>
       </c>
       <c r="C262">
-        <v>45</v>
+        <v>110</v>
       </c>
       <c r="D262">
         <f t="shared" si="4"/>
-        <v>-36445</v>
+        <v>4747</v>
       </c>
     </row>
     <row r="263" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A263" s="1">
-        <v>45183</v>
+        <v>45187</v>
       </c>
       <c r="B263" t="s">
         <v>4</v>
       </c>
       <c r="C263">
-        <v>168</v>
+        <v>192</v>
       </c>
       <c r="D263">
         <f t="shared" si="4"/>
-        <v>-36613</v>
+        <v>4555</v>
       </c>
     </row>
     <row r="264" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A264" s="1">
-        <v>45183</v>
+        <v>45184</v>
       </c>
       <c r="B264" t="s">
         <v>4</v>
       </c>
       <c r="C264">
-        <v>125</v>
+        <v>155</v>
       </c>
       <c r="D264">
         <f t="shared" si="4"/>
-        <v>-36738</v>
+        <v>4400</v>
       </c>
     </row>
     <row r="265" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A265" s="1">
-        <v>45182</v>
+        <v>45184</v>
       </c>
       <c r="B265" t="s">
         <v>4</v>
       </c>
       <c r="C265">
-        <v>92</v>
+        <v>800</v>
       </c>
       <c r="D265">
         <f t="shared" si="4"/>
-        <v>-36830</v>
+        <v>3600</v>
       </c>
     </row>
     <row r="266" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A266" s="1">
-        <v>45182</v>
+        <v>45183</v>
       </c>
       <c r="B266" t="s">
         <v>4</v>
       </c>
       <c r="C266">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="D266">
         <f t="shared" si="4"/>
-        <v>-36920</v>
+        <v>3555</v>
       </c>
     </row>
     <row r="267" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A267" s="1">
-        <v>45181</v>
+        <v>45183</v>
       </c>
       <c r="B267" t="s">
         <v>4</v>
       </c>
       <c r="C267">
-        <v>69</v>
+        <v>168</v>
       </c>
       <c r="D267">
         <f t="shared" si="4"/>
-        <v>-36989</v>
+        <v>3387</v>
       </c>
     </row>
     <row r="268" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A268" s="1">
-        <v>45180</v>
+        <v>45183</v>
       </c>
       <c r="B268" t="s">
         <v>4</v>
       </c>
       <c r="C268">
-        <v>100</v>
+        <v>125</v>
       </c>
       <c r="D268">
         <f t="shared" si="4"/>
-        <v>-37089</v>
+        <v>3262</v>
       </c>
     </row>
     <row r="269" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A269" s="1">
-        <v>45180</v>
+        <v>45182</v>
       </c>
       <c r="B269" t="s">
         <v>4</v>
       </c>
       <c r="C269">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D269">
         <f t="shared" si="4"/>
-        <v>-37184</v>
+        <v>3170</v>
       </c>
     </row>
     <row r="270" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A270" s="1">
-        <v>45180</v>
+        <v>45182</v>
       </c>
       <c r="B270" t="s">
         <v>4</v>
       </c>
       <c r="C270">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="D270">
         <f t="shared" si="4"/>
-        <v>-37254</v>
+        <v>3080</v>
       </c>
     </row>
     <row r="271" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A271" s="1">
-        <v>45180</v>
+        <v>45181</v>
       </c>
       <c r="B271" t="s">
         <v>4</v>
       </c>
       <c r="C271">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="D271">
         <f t="shared" si="4"/>
-        <v>-37334</v>
+        <v>3011</v>
       </c>
     </row>
     <row r="272" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A272" s="1">
-        <v>45177</v>
+        <v>45180</v>
       </c>
       <c r="B272" t="s">
         <v>4</v>
       </c>
       <c r="C272">
-        <v>3000</v>
+        <v>100</v>
       </c>
       <c r="D272">
         <f t="shared" si="4"/>
-        <v>-40334</v>
+        <v>2911</v>
       </c>
     </row>
     <row r="273" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A273" s="1">
-        <v>45176</v>
+        <v>45180</v>
       </c>
       <c r="B273" t="s">
         <v>4</v>
       </c>
       <c r="C273">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="D273">
         <f t="shared" si="4"/>
-        <v>-40434</v>
+        <v>2816</v>
       </c>
     </row>
     <row r="274" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A274" s="1">
-        <v>45176</v>
+        <v>45180</v>
       </c>
       <c r="B274" t="s">
         <v>4</v>
       </c>
       <c r="C274">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="D274">
         <f t="shared" si="4"/>
-        <v>-40534</v>
+        <v>2746</v>
       </c>
     </row>
     <row r="275" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A275" s="1">
-        <v>45175</v>
+        <v>45180</v>
       </c>
       <c r="B275" t="s">
         <v>4</v>
       </c>
       <c r="C275">
-        <v>230</v>
+        <v>80</v>
       </c>
       <c r="D275">
         <f t="shared" si="4"/>
-        <v>-40764</v>
+        <v>2666</v>
       </c>
     </row>
     <row r="276" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A276" s="1">
-        <v>45175</v>
+        <v>45177</v>
       </c>
       <c r="B276" t="s">
         <v>4</v>
       </c>
       <c r="C276">
-        <v>120</v>
+        <v>3000</v>
       </c>
       <c r="D276">
         <f t="shared" si="4"/>
-        <v>-40884</v>
+        <v>-334</v>
       </c>
     </row>
     <row r="277" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A277" s="1">
-        <v>45175</v>
+        <v>45176</v>
       </c>
       <c r="B277" t="s">
         <v>4</v>
       </c>
       <c r="C277">
-        <v>158</v>
+        <v>100</v>
       </c>
       <c r="D277">
         <f t="shared" si="4"/>
-        <v>-41042</v>
+        <v>-434</v>
       </c>
     </row>
     <row r="278" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A278" s="1">
-        <v>45174</v>
+        <v>45176</v>
       </c>
       <c r="B278" t="s">
         <v>4</v>
       </c>
       <c r="C278">
-        <v>226</v>
+        <v>100</v>
       </c>
       <c r="D278">
         <f t="shared" si="4"/>
-        <v>-41268</v>
+        <v>-534</v>
       </c>
     </row>
     <row r="279" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A279" s="1">
-        <v>45167</v>
+        <v>45175</v>
       </c>
       <c r="B279" t="s">
         <v>4</v>
       </c>
       <c r="C279">
-        <v>1200</v>
+        <v>230</v>
       </c>
       <c r="D279">
         <f t="shared" si="4"/>
-        <v>-42468</v>
+        <v>-764</v>
       </c>
     </row>
     <row r="280" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A280" s="1">
-        <v>45167</v>
+        <v>45175</v>
       </c>
       <c r="B280" t="s">
         <v>4</v>
@@ -4644,22 +4648,97 @@
       </c>
       <c r="D280">
         <f t="shared" si="4"/>
-        <v>-42588</v>
+        <v>-884</v>
       </c>
     </row>
     <row r="281" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A281" s="1">
-        <v>45167</v>
+        <v>45175</v>
       </c>
       <c r="B281" t="s">
         <v>4</v>
       </c>
       <c r="C281">
-        <v>700</v>
+        <v>158</v>
       </c>
       <c r="D281">
         <f t="shared" si="4"/>
-        <v>-43288</v>
+        <v>-1042</v>
+      </c>
+    </row>
+    <row r="282" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A282" s="1">
+        <v>45174</v>
+      </c>
+      <c r="B282" t="s">
+        <v>4</v>
+      </c>
+      <c r="C282">
+        <v>226</v>
+      </c>
+      <c r="D282">
+        <f t="shared" si="4"/>
+        <v>-1268</v>
+      </c>
+    </row>
+    <row r="283" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A283" s="1">
+        <v>45170</v>
+      </c>
+      <c r="B283" t="s">
+        <v>5</v>
+      </c>
+      <c r="C283">
+        <v>10000</v>
+      </c>
+      <c r="D283">
+        <f t="shared" si="4"/>
+        <v>8732</v>
+      </c>
+    </row>
+    <row r="284" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A284" s="1">
+        <v>45167</v>
+      </c>
+      <c r="B284" t="s">
+        <v>4</v>
+      </c>
+      <c r="C284">
+        <v>1200</v>
+      </c>
+      <c r="D284">
+        <f t="shared" si="4"/>
+        <v>7532</v>
+      </c>
+    </row>
+    <row r="285" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A285" s="1">
+        <v>45167</v>
+      </c>
+      <c r="B285" t="s">
+        <v>4</v>
+      </c>
+      <c r="C285">
+        <v>120</v>
+      </c>
+      <c r="D285">
+        <f t="shared" si="4"/>
+        <v>7412</v>
+      </c>
+    </row>
+    <row r="286" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A286" s="1">
+        <v>45167</v>
+      </c>
+      <c r="B286" t="s">
+        <v>4</v>
+      </c>
+      <c r="C286">
+        <v>700</v>
+      </c>
+      <c r="D286">
+        <f t="shared" si="4"/>
+        <v>6712</v>
       </c>
     </row>
   </sheetData>

</xml_diff>